<commit_message>
feat: add RS232 SCPI power supply acceptance
</commit_message>
<xml_diff>
--- a/Workflows/real-device-acceptance.xlsx
+++ b/Workflows/real-device-acceptance.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品追溯信息表" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试工步表'!$A$1:$P$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试工步表'!$A$1:$P$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -561,43 +561,39 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DoIP</t>
+          <t>电源</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>DoIP_ECU</t>
+          <t>DC_Power_Supply</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TCP:13400</t>
+          <t>COM3</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>DiagnosticSessionControl 10 01</t>
+          <t>RS232 SCPI DC Power Supply ON</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>send_uds</t>
+          <t>power_on</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>host=192.168.0.100,port=13400,sourceAddress=0x102D,targetAddress=0x1008,activationType=0x00,udsPayload=10 01,expectedPrefix=50 01,connectionMode=session</t>
+          <t>port=COM3,baudRate=9600,dataBits=8,stopBits=1,parity=N,voltage=12.0,current=1.0,powerOnDelayMs=1000</t>
         </is>
       </c>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
       <c r="J2" s="2" t="n"/>
       <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>hex</t>
-        </is>
-      </c>
+      <c r="L2" s="2" t="n"/>
       <c r="M2" s="2" t="n">
         <v>5000</v>
       </c>
@@ -608,7 +604,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>替换 ECU IP、逻辑地址和 UDS 期望响应</t>
+          <t>替换 COM 口、电压、电流和上电稳定时间</t>
         </is>
       </c>
       <c r="P2" s="2" t="n"/>
@@ -619,45 +615,41 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Modbus</t>
+          <t>DoIP</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Modbus_PLC</t>
+          <t>DoIP_ECU</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>TCP:502</t>
+          <t>TCP:13400</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Read Holding Register 0</t>
+          <t>DiagnosticSessionControl 10 01</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>read</t>
+          <t>send_uds</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>transport=tcp,host=192.168.0.101,port=502,slaveId=1,functionCode=3,startAddr=0,quantity=1,valueType=uint16,valueOffset=0,valueLength=2</t>
+          <t>host=192.168.0.100,port=13400,sourceAddress=0x102D,targetAddress=0x1008,activationType=0x00,udsPayload=10 01,expectedPrefix=50 01,connectionMode=session</t>
         </is>
       </c>
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="2" t="n">
-        <v>65535</v>
-      </c>
+      <c r="J3" s="2" t="n"/>
+      <c r="K3" s="2" t="n"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>counts</t>
+          <t>hex</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
@@ -670,14 +662,10 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>替换寄存器地址、从站号和工程限值</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>[{"name": "register_value", "offset": 0, "length": 2, "type": "uint16", "endian": "big", "unit": "counts"}]</t>
-        </is>
-      </c>
+          <t>替换 ECU IP、逻辑地址和 UDS 期望响应</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -685,49 +673,45 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SCPI</t>
+          <t>Modbus</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>SCPI_DMM</t>
+          <t>Modbus_PLC</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>TCP:5025</t>
+          <t>TCP:502</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Instrument Identification</t>
+          <t>Read Holding Register 0</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>*IDN?</t>
+          <t>read</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>scpi.idn</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>.+</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>5000</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
+          <t>transport=tcp,host=192.168.0.101,port=502,slaveId=1,functionCode=3,startAddr=0,quantity=1,valueType=uint16,valueOffset=0,valueLength=2</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>65535</v>
+      </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>counts</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
@@ -735,15 +719,19 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>停机</t>
+          <t>重试1次</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>确认仪器返回非空身份信息</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="n"/>
+          <t>替换寄存器地址、从站号和工程限值</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>[{"name": "register_value", "offset": 0, "length": 2, "type": "uint16", "endian": "big", "unit": "counts"}]</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -766,22 +754,22 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>DC Voltage</t>
+          <t>Instrument Identification</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>MEAS:VOLT:DC?</t>
+          <t>*IDN?</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>scpi.voltage</t>
+          <t>scpi.idn</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[-+0-9.eE]+</t>
+          <t>.+</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -789,15 +777,11 @@
           <t>5000</t>
         </is>
       </c>
-      <c r="J5" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="2" t="n">
-        <v>1000</v>
-      </c>
+      <c r="J5" s="2" t="n"/>
+      <c r="K5" s="2" t="n"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>text</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
@@ -810,17 +794,141 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
+          <t>确认仪器返回非空身份信息</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>SCPI</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>SCPI_DMM</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>TCP:5025</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>DC Voltage</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>MEAS:VOLT:DC?</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>scpi.voltage</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>[-+0-9.eE]+</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>停机</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
           <t>将上下限改为 DUT 规格；默认范围仅用于连通性验证</t>
         </is>
       </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>[{"name": "scpi_value", "type": "double", "unit": "V", "trim": true}]</t>
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>电源</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>DC_Power_Supply</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>COM3</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>RS232 SCPI DC Power Supply OFF</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>power_off</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>port=COM3,baudRate=9600,dataBits=8,stopBits=1,parity=N</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>继续</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>确认测试完成后关闭输出</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P5"/>
+  <autoFilter ref="A1:P7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -831,7 +939,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -934,40 +1042,34 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>DoIP</t>
+          <t>电源</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>DoIP_ECU</t>
+          <t>DC_Power_Supply</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TCP:13400</t>
+          <t>COM3</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>TCP</t>
+          <t>串口</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>192.168.0.100</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>13400</v>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>0x1008</t>
-        </is>
-      </c>
+          <t>COM3</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>DUT DoIP Gateway</t>
+          <t>SCPI DC Power Supply</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -975,9 +1077,17 @@
           <t>TODO</t>
         </is>
       </c>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
+      <c r="K2" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
           <t>是</t>
@@ -985,7 +1095,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>修改为实际 ECU 地址</t>
+          <t>确认 RS232 电源串口和 SCPI 终止符</t>
         </is>
       </c>
     </row>
@@ -995,17 +1105,17 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Modbus</t>
+          <t>DoIP</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Modbus_PLC</t>
+          <t>DoIP_ECU</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>TCP:502</t>
+          <t>TCP:13400</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1015,18 +1125,20 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>192.168.0.101</t>
+          <t>192.168.0.100</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
-        <v>502</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>1</v>
+        <v>13400</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>0x1008</t>
+        </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>PLC/Device</t>
+          <t>DUT DoIP Gateway</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1044,7 +1156,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>修改为实际从站和寄存器映射</t>
+          <t>修改为实际 ECU 地址</t>
         </is>
       </c>
     </row>
@@ -1054,17 +1166,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SCPI</t>
+          <t>Modbus</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>SCPI_DMM</t>
+          <t>Modbus_PLC</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>TCP:5025</t>
+          <t>TCP:502</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1074,16 +1186,18 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>192.168.0.102</t>
+          <t>192.168.0.101</t>
         </is>
       </c>
       <c r="G4" s="2" t="n">
-        <v>5025</v>
-      </c>
-      <c r="H4" s="2" t="n"/>
+        <v>502</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>DMM</t>
+          <t>PLC/Device</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -1100,6 +1214,63 @@
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>修改为实际从站和寄存器映射</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>SCPI</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>SCPI_DMM</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>TCP:5025</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>TCP</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>192.168.0.102</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>5025</v>
+      </c>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>DMM</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>TODO</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="n"/>
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="n"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>确认仪器已开启远程控制</t>
         </is>
@@ -1251,7 +1422,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>已替换所有 TODO、IP、地址和上下限</t>
+          <t>已替换所有 TODO、COM 口、IP、地址和上下限</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
refactor: use English acceptance configuration values
</commit_message>
<xml_diff>
--- a/Workflows/real-device-acceptance.xlsx
+++ b/Workflows/real-device-acceptance.xlsx
@@ -561,7 +561,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>电源</t>
+          <t>PowerSupply</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>重试1次</t>
+          <t>retry 1</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -657,7 +657,7 @@
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>重试1次</t>
+          <t>retry 1</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>重试1次</t>
+          <t>retry 1</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>停机</t>
+          <t>fail_fast</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>停机</t>
+          <t>fail_fast</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
@@ -879,7 +879,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>电源</t>
+          <t>PowerSupply</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -917,7 +917,7 @@
       </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>继续</t>
+          <t>continue</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>电源</t>
+          <t>PowerSupply</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>串口</t>
+          <t>Serial</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1090,7 +1090,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -1151,7 +1151,7 @@
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
@@ -1210,7 +1210,7 @@
       <c r="M4" s="2" t="n"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
refactor: decouple device types from plugin IDs
</commit_message>
<xml_diff>
--- a/Workflows/real-device-acceptance.xlsx
+++ b/Workflows/real-device-acceptance.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品追溯信息表" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试工步表'!$A$1:$P$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'测试工步表'!$A$1:$Q$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -471,6 +471,7 @@
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="72" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -552,6 +553,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>解码配置</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Plugin ID</t>
         </is>
       </c>
     </row>
@@ -608,6 +614,11 @@
         </is>
       </c>
       <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>power.supply</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -666,6 +677,11 @@
         </is>
       </c>
       <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>doip.master</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -732,6 +748,11 @@
           <t>[{"name": "register_value", "offset": 0, "length": 2, "type": "uint16", "endian": "big", "unit": "counts"}]</t>
         </is>
       </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>modbus.master</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -739,7 +760,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SCPI</t>
+          <t>Multimeter</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -798,6 +819,11 @@
         </is>
       </c>
       <c r="P5" s="2" t="n"/>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>scpi.command</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -805,7 +831,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SCPI</t>
+          <t>Multimeter</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -870,6 +896,11 @@
       <c r="P6" s="2" t="inlineStr">
         <is>
           <t>[{"name": "scpi_value", "type": "double", "unit": "V", "trim": true}]</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>scpi.command</t>
         </is>
       </c>
     </row>
@@ -926,9 +957,14 @@
         </is>
       </c>
       <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>power.supply</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P7"/>
+  <autoFilter ref="A1:Q7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>